<commit_message>
change db.sql,  push temp function createWithUploadQuestion in test.service.js
</commit_message>
<xml_diff>
--- a/documents/parts-insert-base.xlsx
+++ b/documents/parts-insert-base.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>partName</t>
   </si>
@@ -43,6 +43,9 @@
   </si>
   <si>
     <t>Part 7</t>
+  </si>
+  <si>
+    <t>partNumber</t>
   </si>
 </sst>
 </file>
@@ -368,49 +371,73 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8">
         <v>7</v>
       </c>
     </row>

</xml_diff>